<commit_message>
docs: update full ss9
</commit_message>
<xml_diff>
--- a/JPD/documents/full_jpd.xlsx
+++ b/JPD/documents/full_jpd.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fptu\JPD\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2AE732-036A-4190-B3BC-7782359E3A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6B7598-3B9D-490D-AD7F-9498D3B5CBB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{FA3ADD2E-6701-4EA2-BF3C-245AE1375C42}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="278">
   <si>
     <t>イベント</t>
   </si>
@@ -592,13 +592,347 @@
   </si>
   <si>
     <t>だけ</t>
+  </si>
+  <si>
+    <t>例：</t>
+  </si>
+  <si>
+    <t>あさ、ジョギングをして、シャクーをあびて、かいしゃへ行きます。</t>
+  </si>
+  <si>
+    <t>Ｖて、それから。。。Ｖました。</t>
+  </si>
+  <si>
+    <t>Ｖ１て、Ｖ２て、。。。Ｖます/ました。</t>
+  </si>
+  <si>
+    <t>昨日、６じにおきて、ジョギングをして、それからあさごはんを食べました。</t>
+  </si>
+  <si>
+    <t>どうやってＶますか。</t>
+  </si>
+  <si>
+    <t>LIÊN KẾT ĐỘNG TỪ「どうし」</t>
+  </si>
+  <si>
+    <t>LIỆT KÊ HÀNH ĐỘNG</t>
+  </si>
+  <si>
+    <t>→ LÀM CÁCH NÀO ĐỂ LÀM「 V1」?</t>
+  </si>
+  <si>
+    <t>→Ｖ１て、Ｖ２て、。。。Ｖます。</t>
+  </si>
+  <si>
+    <t>→ TÔI ĐÃ LÀM 「V1」RỒI LÀM「 V2」。。。LÀM「 V」</t>
+  </si>
+  <si>
+    <t>ーどうやってきっぷを買いますか。</t>
+  </si>
+  <si>
+    <t>Làm cách nào để mua vé ạ?</t>
+  </si>
+  <si>
+    <t>Xin hãy cho tiền vào đây, rồi ấn cái nút này.</t>
+  </si>
+  <si>
+    <t>ーここにおかねをいれて、このボタンをおしてください。</t>
+  </si>
+  <si>
+    <t>漢字</t>
+  </si>
+  <si>
+    <t>好 HẢO</t>
+  </si>
+  <si>
+    <t>外国　「がいこく」　nước ngoài</t>
+  </si>
+  <si>
+    <t>外国語　「がいこくご」　ngoại ngữ</t>
+  </si>
+  <si>
+    <t>文法</t>
+  </si>
+  <si>
+    <t>好き(な)　「すきな」　thích</t>
+  </si>
+  <si>
+    <t>大好き　「だいすき」　rất thích</t>
+  </si>
+  <si>
+    <t>大好物　「だいこうぶつ」　món yêu thích</t>
+  </si>
+  <si>
+    <t>歌 CA</t>
+  </si>
+  <si>
+    <t>歌　「うた」bài hát</t>
+  </si>
+  <si>
+    <t>歌う　「うたう」　hát</t>
+  </si>
+  <si>
+    <t>国歌　「こっか」　Quốc ca</t>
+  </si>
+  <si>
+    <t>短歌　「たんか」　thơ ngắn</t>
+  </si>
+  <si>
+    <t>音 ÂM</t>
+  </si>
+  <si>
+    <t>音　「おと」　âm thanh</t>
+  </si>
+  <si>
+    <t>音読み　「お   んよみ」　âm On</t>
+  </si>
+  <si>
+    <t>楽 NHẠC, LẠC</t>
+  </si>
+  <si>
+    <t>楽しい　「たのしい」　vui vẻ</t>
+  </si>
+  <si>
+    <t>音楽　「おんがく」　âm nhạc</t>
+  </si>
+  <si>
+    <t>車 XA</t>
+  </si>
+  <si>
+    <t>車　「くるま」　xe hơi</t>
+  </si>
+  <si>
+    <t>映 ẢNH, ÁNH</t>
+  </si>
+  <si>
+    <t>映画　「えいが」　phim</t>
+  </si>
+  <si>
+    <t>画 HỌA, HOẠCH</t>
+  </si>
+  <si>
+    <t>計画　「けいかく」　　kế hoạch, dự án</t>
+  </si>
+  <si>
+    <t>旅 LỮ</t>
+  </si>
+  <si>
+    <t>旅　「たび」　chuyến đi, du lịch, cuộc hành trình</t>
+  </si>
+  <si>
+    <t>旅行　「りょこう」　du lịch</t>
+  </si>
+  <si>
+    <t>海 HẢI</t>
+  </si>
+  <si>
+    <t>海　「うみ」　biển</t>
+  </si>
+  <si>
+    <t>海水　「かいすい」　nước biển</t>
+  </si>
+  <si>
+    <t>外 NGOẠI, NGOÀI</t>
+  </si>
+  <si>
+    <t>家の外　「いえのそと」　bên ngoài nhà</t>
+  </si>
+  <si>
+    <t>外国人　「がいこくじん」　người nước ngoài</t>
+  </si>
+  <si>
+    <t>社外　「しゃがい」　ngoài công ty, bên ngoài doanh nghiệp</t>
+  </si>
+  <si>
+    <t>海外　「かいがい」　hải ngoại, ngước ngoài</t>
+  </si>
+  <si>
+    <t>辞書形　「Ｖる」：Thể nguyên dạng (từ điển) của động từ</t>
+  </si>
+  <si>
+    <t>「じしょけ」 là dạng ngắn của 「Ｖます」</t>
+  </si>
+  <si>
+    <t>Ｖます　→　Ｖる</t>
+  </si>
+  <si>
+    <t>Động từ nhóm 3 「三グループ」</t>
+  </si>
+  <si>
+    <t>Động từ nhóm 2 「ニグループ」</t>
+  </si>
+  <si>
+    <t>Động từ nhóm 1 「一グループ」</t>
+  </si>
+  <si>
+    <t>来ます→くる</t>
+  </si>
+  <si>
+    <t>します→する</t>
+  </si>
+  <si>
+    <t>食べます→食べる</t>
+  </si>
+  <si>
+    <t>見ます→見る</t>
+  </si>
+  <si>
+    <r>
+      <t>Ｖ</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Mincho"/>
+        <family val="1"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ます</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Mincho"/>
+        <family val="1"/>
+        <charset val="128"/>
+      </rPr>
+      <t>＋る→Ｖる</t>
+    </r>
+  </si>
+  <si>
+    <t>～います→う</t>
+  </si>
+  <si>
+    <r>
+      <t>～い</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Mincho"/>
+        <family val="1"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ます</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Mincho"/>
+        <family val="1"/>
+        <charset val="128"/>
+      </rPr>
+      <t>→う</t>
+    </r>
+  </si>
+  <si>
+    <t>～きます→く</t>
+  </si>
+  <si>
+    <t>～ぎます→ぐ</t>
+  </si>
+  <si>
+    <t>～します→す</t>
+  </si>
+  <si>
+    <t>～ちます→つ</t>
+  </si>
+  <si>
+    <t>～にます→ぬ</t>
+  </si>
+  <si>
+    <t>～みます→む</t>
+  </si>
+  <si>
+    <t>～びます→ぶ</t>
+  </si>
+  <si>
+    <t>～ります→る</t>
+  </si>
+  <si>
+    <t>私のしゅみは　N/Vること　です。</t>
+  </si>
+  <si>
+    <t>私のしゅみはまんがをよむことです。</t>
+  </si>
+  <si>
+    <t>私のしゅみはおんがくをきくことです。</t>
+  </si>
+  <si>
+    <t>あなたのしゅみは何ですか。</t>
+  </si>
+  <si>
+    <t>→ Sở thích của tôi là 「N/V」</t>
+  </si>
+  <si>
+    <t>→ Sở thích của bạn là gì?</t>
+  </si>
+  <si>
+    <t>Từ số lượng　に　Lượng từ</t>
+  </si>
+  <si>
+    <t>(Chỉ thời gian) (Số lượng/ Số lần)</t>
+  </si>
+  <si>
+    <t>Cách nói dùng để chỉ tần suất</t>
+  </si>
+  <si>
+    <t>一週間に一回映画がみます。</t>
+  </si>
+  <si>
+    <t>一週間に2，3冊本が読みます。</t>
+  </si>
+  <si>
+    <t>Khả năng, năng lực:</t>
+  </si>
+  <si>
+    <t>N/Vること　が　できます/できません。</t>
+  </si>
+  <si>
+    <t>毎日、食べることができます。</t>
+  </si>
+  <si>
+    <t>ミラーさんは日本語ができます。</t>
+  </si>
+  <si>
+    <t>→ Có thể (có khả năng) làm 「N/V」</t>
+  </si>
+  <si>
+    <t>なかなか～ができません。</t>
+  </si>
+  <si>
+    <t>日本でなかなかうまをみることができません。</t>
+  </si>
+  <si>
+    <t>ひらがなをかくことができますか。</t>
+  </si>
+  <si>
+    <t>ーはい、できます。</t>
+  </si>
+  <si>
+    <t>ーいいえ、できません。</t>
+  </si>
+  <si>
+    <t>N/Ｖること　が　できますか。</t>
+  </si>
+  <si>
+    <t>→ Mãi mà không thể…/ Khó mà có thể…</t>
+  </si>
+  <si>
+    <t>→ Có thể làm 「V」 không?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -608,12 +942,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Cambria"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -621,13 +949,28 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Mincho"/>
+      <family val="1"/>
+      <charset val="128"/>
+    </font>
+    <font>
       <b/>
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Yu Mincho"/>
+      <family val="1"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Mincho"/>
+      <family val="1"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -702,13 +1045,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -718,8 +1057,54 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1145,943 +1530,1747 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FF088B7-57DB-42FE-8A82-081056E8782F}">
-  <dimension ref="A1:D77"/>
+  <dimension ref="A2:U82"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.5546875" customWidth="1"/>
-    <col min="2" max="2" width="29.21875" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="41" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18" style="1" customWidth="1"/>
+    <col min="4" max="4" width="41" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="8"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
+      <c r="F2" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="13"/>
+      <c r="N2" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="F3" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="G3" s="6"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="8"/>
+      <c r="N3" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="F4" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="13"/>
+      <c r="N4" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="F5" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="13"/>
+      <c r="N5" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="5"/>
+      <c r="D6" s="5" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="F6" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="13"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="5"/>
+      <c r="D7" s="5" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="F7" s="6"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="8"/>
+      <c r="N7" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="F8" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="8"/>
+      <c r="N8" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+      <c r="F9" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="13"/>
+      <c r="N9" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
         <v>8</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="F10" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="13"/>
+      <c r="N10" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
         <v>9</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
+      <c r="F11" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="13"/>
+      <c r="N11" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
         <v>10</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="5"/>
+      <c r="D12" s="5" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
+      <c r="F12" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="18"/>
+      <c r="N12" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
         <v>11</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="F13" s="6"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="8"/>
+      <c r="N13" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" s="5">
         <v>12</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
+      <c r="F14" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="8"/>
+      <c r="N14" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="5">
         <v>13</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
+      <c r="F15" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="13"/>
+      <c r="N15" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="5">
         <v>14</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
+      <c r="F16" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="13"/>
+      <c r="N16" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
         <v>15</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
+      <c r="F17" s="6"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="8"/>
+      <c r="N17" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
         <v>16</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
+      <c r="F18" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="G18" s="5"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="8"/>
+      <c r="N18" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
         <v>17</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="2">
+      <c r="F19" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="13"/>
+      <c r="N19" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" s="5">
         <v>18</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
+      <c r="F20" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="13"/>
+      <c r="N20" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="5">
         <v>19</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
+      <c r="F21" s="6"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="8"/>
+      <c r="N21" s="1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="5">
         <v>20</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2" t="s">
+      <c r="F22" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="G22" s="6"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="8"/>
+      <c r="N22" s="1" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="5"/>
+      <c r="D23" s="5" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
+      <c r="F23" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="13"/>
+      <c r="N23" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A24" s="5">
         <v>21</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="2">
+      <c r="F24" s="6"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="8"/>
+      <c r="N24" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A25" s="5">
         <v>22</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="5" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
+      <c r="F25" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="G25" s="5"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="8"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="5">
         <v>23</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
+      <c r="F26" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="13"/>
+      <c r="N26" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="5">
         <v>24</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="5" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="2">
+      <c r="F27" s="6"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="8"/>
+      <c r="N27" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" s="5">
         <v>25</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="2">
+      <c r="F28" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="G28" s="5"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="8"/>
+      <c r="N28" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A29" s="5">
         <v>26</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="5" t="s">
+      <c r="C29" s="5"/>
+      <c r="D29" s="9" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
+      <c r="F29" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="13"/>
+      <c r="N29" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A30" s="5">
         <v>27</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="5" t="s">
+      <c r="C30" s="5"/>
+      <c r="D30" s="9" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2" t="s">
+      <c r="F30" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="13"/>
+      <c r="N30" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="5" t="s">
+      <c r="C31" s="5"/>
+      <c r="D31" s="9" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="2">
+      <c r="F31" s="6"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="8"/>
+      <c r="N31" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="5">
         <v>28</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="5" t="s">
+      <c r="C32" s="5"/>
+      <c r="D32" s="9" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="2">
+      <c r="F32" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="G32" s="6"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="7"/>
+      <c r="L32" s="8"/>
+      <c r="N32" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" s="5">
         <v>29</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="5" t="s">
+      <c r="C33" s="5"/>
+      <c r="D33" s="9" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2" t="s">
+      <c r="F33" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="13"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="5" t="s">
+      <c r="C34" s="5"/>
+      <c r="D34" s="9" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
+      <c r="F34" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="13"/>
+      <c r="N34" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A35" s="5">
         <v>30</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="9" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="3">
+      <c r="F35" s="6"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="8"/>
+      <c r="N35" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" s="9">
         <v>31</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="5" t="s">
+      <c r="C36" s="5"/>
+      <c r="D36" s="9" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="2">
+      <c r="F36" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="G36" s="6"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="7"/>
+      <c r="K36" s="7"/>
+      <c r="L36" s="8"/>
+      <c r="N36" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A37" s="5">
         <v>32</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="5" t="s">
+      <c r="C37" s="5"/>
+      <c r="D37" s="9" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="s">
+      <c r="F37" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="13"/>
+      <c r="N37" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="F38" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="12"/>
+      <c r="L38" s="13"/>
+      <c r="N38" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="F39" s="6"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="7"/>
+      <c r="K39" s="7"/>
+      <c r="L39" s="8"/>
+      <c r="N39" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="8"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="2">
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="4"/>
+      <c r="F40" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="7"/>
+      <c r="L40" s="8"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A41" s="5">
         <v>1</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="4" t="s">
+      <c r="C41" s="5"/>
+      <c r="D41" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="2">
+      <c r="F41" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="13"/>
+      <c r="N41" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A42" s="5">
         <v>2</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C42" s="2"/>
-      <c r="D42" s="4" t="s">
+      <c r="C42" s="5"/>
+      <c r="D42" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="2">
+      <c r="F42" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="13"/>
+      <c r="N42" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" s="5">
         <v>3</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D43" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="2">
+      <c r="F43" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="12"/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="12"/>
+      <c r="L43" s="13"/>
+      <c r="N43" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A44" s="5">
         <v>4</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C44" s="2"/>
-      <c r="D44" s="4" t="s">
+      <c r="C44" s="5"/>
+      <c r="D44" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="2">
+      <c r="F44" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="12"/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="12"/>
+      <c r="L44" s="13"/>
+      <c r="N44" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" s="5">
         <v>5</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="4" t="s">
+      <c r="C45" s="5"/>
+      <c r="D45" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="2">
+      <c r="F45" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="13"/>
+      <c r="N45" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" s="5">
         <v>6</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C46" s="2"/>
-      <c r="D46" s="4" t="s">
+      <c r="C46" s="5"/>
+      <c r="D46" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2" t="s">
+      <c r="F46" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12"/>
+      <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
+      <c r="L46" s="13"/>
+      <c r="N46" s="1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="4" t="s">
+      <c r="C47" s="5"/>
+      <c r="D47" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="2">
+      <c r="N47" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" s="5">
         <v>7</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C48" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D48" s="4" t="s">
+      <c r="D48" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2" t="s">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="4" t="s">
+      <c r="C49" s="5"/>
+      <c r="D49" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="2">
+      <c r="N49" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A50" s="5">
         <v>8</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="D50" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="2">
+      <c r="N50" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="O50" s="19"/>
+      <c r="P50" s="19"/>
+      <c r="Q50" s="19"/>
+      <c r="R50" s="19"/>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A51" s="5">
         <v>9</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D51" s="4" t="s">
+      <c r="D51" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="2">
+      <c r="N51" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A52" s="5">
         <v>10</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="C52" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D52" s="4" t="s">
+      <c r="D52" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2" t="s">
+      <c r="N52" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A53" s="5"/>
+      <c r="B53" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C53" s="2"/>
-      <c r="D53" s="4" t="s">
+      <c r="C53" s="5"/>
+      <c r="D53" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="2">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A54" s="5">
         <v>11</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="D54" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="2">
+      <c r="N54" s="1" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A55" s="5">
         <v>12</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C55" s="2"/>
-      <c r="D55" s="4" t="s">
+      <c r="C55" s="5"/>
+      <c r="D55" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2" t="s">
+      <c r="N55" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A56" s="5"/>
+      <c r="B56" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="4" t="s">
+      <c r="C56" s="5"/>
+      <c r="D56" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" s="2">
+      <c r="N56" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A57" s="5">
         <v>13</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C57" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="D57" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="2">
+      <c r="N57" s="1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A58" s="5">
         <v>14</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C58" s="2"/>
-      <c r="D58" s="4" t="s">
+      <c r="C58" s="5"/>
+      <c r="D58" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="2">
+      <c r="N58" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A59" s="5">
         <v>15</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C59" s="2"/>
-      <c r="D59" s="4" t="s">
+      <c r="C59" s="5"/>
+      <c r="D59" s="5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="2">
+      <c r="N59" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A60" s="5">
         <v>16</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D60" s="4" t="s">
+      <c r="D60" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="9" t="s">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="N62" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A63" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="2">
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
+      <c r="N63" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="O63" s="20"/>
+      <c r="P63" s="20"/>
+      <c r="Q63" s="20"/>
+      <c r="R63" s="20"/>
+      <c r="S63" s="20"/>
+      <c r="T63" s="20"/>
+      <c r="U63" s="20"/>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A64" s="5">
         <v>1</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C64" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D64" s="4" t="s">
+      <c r="D64" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="2">
+      <c r="N64" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="O64" s="21"/>
+      <c r="P64" s="21"/>
+      <c r="Q64" s="21"/>
+      <c r="R64" s="21"/>
+      <c r="S64" s="21"/>
+      <c r="T64" s="21"/>
+      <c r="U64" s="21"/>
+    </row>
+    <row r="65" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A65" s="5">
         <v>2</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C65" s="2"/>
-      <c r="D65" s="4" t="s">
+      <c r="C65" s="5"/>
+      <c r="D65" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2" t="s">
+      <c r="N65" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="O65" s="20"/>
+      <c r="P65" s="20"/>
+      <c r="Q65" s="20"/>
+      <c r="R65" s="20"/>
+      <c r="S65" s="20"/>
+      <c r="T65" s="20"/>
+      <c r="U65" s="20"/>
+    </row>
+    <row r="66" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D66" s="4" t="s">
+      <c r="D66" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="2">
+      <c r="N66" s="21"/>
+      <c r="O66" s="21"/>
+      <c r="P66" s="21"/>
+      <c r="Q66" s="21"/>
+      <c r="R66" s="21"/>
+      <c r="S66" s="21"/>
+      <c r="T66" s="21"/>
+      <c r="U66" s="21"/>
+    </row>
+    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A67" s="5">
         <v>3</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D67" s="4" t="s">
+      <c r="D67" s="5" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="2">
+      <c r="N67" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="O67" s="20"/>
+      <c r="P67" s="20"/>
+      <c r="Q67" s="20"/>
+      <c r="R67" s="20"/>
+      <c r="S67" s="20"/>
+      <c r="T67" s="20"/>
+      <c r="U67" s="21"/>
+    </row>
+    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A68" s="5">
         <v>4</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="C68" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D68" s="4" t="s">
+      <c r="D68" s="5" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="2">
+      <c r="N68" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="O68" s="21"/>
+      <c r="P68" s="21"/>
+      <c r="Q68" s="21"/>
+      <c r="R68" s="21"/>
+      <c r="S68" s="21"/>
+      <c r="T68" s="21"/>
+      <c r="U68" s="21"/>
+    </row>
+    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A69" s="5">
         <v>5</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D69" s="4" t="s">
+      <c r="D69" s="5" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="2">
+      <c r="N69" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="O69" s="21"/>
+      <c r="P69" s="21"/>
+      <c r="Q69" s="21"/>
+      <c r="R69" s="21"/>
+      <c r="S69" s="21"/>
+      <c r="T69" s="21"/>
+      <c r="U69" s="22"/>
+    </row>
+    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A70" s="5">
         <v>6</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D70" s="4" t="s">
+      <c r="D70" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="2">
+      <c r="N70" s="21"/>
+      <c r="O70" s="21"/>
+      <c r="P70" s="21"/>
+      <c r="Q70" s="21"/>
+      <c r="R70" s="21"/>
+      <c r="S70" s="21"/>
+      <c r="T70" s="21"/>
+      <c r="U70" s="21"/>
+    </row>
+    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A71" s="5">
         <v>7</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="C71" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D71" s="4" t="s">
+      <c r="D71" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="2">
+      <c r="N71" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="O71" s="21"/>
+      <c r="P71" s="21"/>
+      <c r="Q71" s="21"/>
+      <c r="R71" s="21"/>
+      <c r="S71" s="21"/>
+      <c r="T71" s="21"/>
+      <c r="U71" s="21"/>
+    </row>
+    <row r="72" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A72" s="5">
         <v>8</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C72" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D72" s="4" t="s">
+      <c r="D72" s="5" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="2">
+      <c r="N72" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="O72" s="21"/>
+      <c r="P72" s="21"/>
+      <c r="Q72" s="21"/>
+      <c r="R72" s="21"/>
+      <c r="S72" s="21"/>
+      <c r="T72" s="21"/>
+      <c r="U72" s="21"/>
+    </row>
+    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A73" s="5">
         <v>9</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C73" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D73" s="4" t="s">
+      <c r="D73" s="5" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="2">
+      <c r="N73" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="O73" s="21"/>
+      <c r="P73" s="21"/>
+      <c r="Q73" s="21"/>
+      <c r="R73" s="21"/>
+      <c r="S73" s="21"/>
+      <c r="T73" s="21"/>
+      <c r="U73" s="21"/>
+    </row>
+    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A74" s="5">
         <v>10</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C74" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D74" s="4" t="s">
+      <c r="D74" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="2">
+      <c r="N74" s="21"/>
+      <c r="O74" s="21"/>
+      <c r="P74" s="21"/>
+      <c r="Q74" s="21"/>
+      <c r="R74" s="21"/>
+      <c r="S74" s="21"/>
+      <c r="T74" s="21"/>
+      <c r="U74" s="21"/>
+    </row>
+    <row r="75" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A75" s="5">
         <v>11</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C75" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D75" s="4" t="s">
+      <c r="D75" s="5" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="2">
+      <c r="N75" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="O75" s="20"/>
+      <c r="P75" s="20"/>
+      <c r="Q75" s="20"/>
+      <c r="R75" s="20"/>
+      <c r="S75" s="20"/>
+      <c r="T75" s="20"/>
+      <c r="U75" s="20"/>
+    </row>
+    <row r="76" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A76" s="5">
         <v>12</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C76" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D76" s="4" t="s">
+      <c r="D76" s="5" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="2">
+      <c r="N76" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="O76" s="20"/>
+      <c r="P76" s="20"/>
+      <c r="Q76" s="20"/>
+      <c r="R76" s="20"/>
+      <c r="S76" s="20"/>
+      <c r="T76" s="20"/>
+      <c r="U76" s="20"/>
+    </row>
+    <row r="77" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A77" s="5">
         <v>13</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C77" s="2"/>
-      <c r="D77" s="4" t="s">
+      <c r="C77" s="5"/>
+      <c r="D77" s="5" t="s">
         <v>73</v>
       </c>
+      <c r="N77" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="O77" s="20"/>
+      <c r="P77" s="20"/>
+      <c r="Q77" s="20"/>
+      <c r="R77" s="20"/>
+      <c r="S77" s="20"/>
+      <c r="T77" s="20"/>
+      <c r="U77" s="20"/>
+    </row>
+    <row r="78" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="N78" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="O78" s="21"/>
+      <c r="P78" s="21"/>
+      <c r="Q78" s="21"/>
+      <c r="R78" s="21"/>
+      <c r="S78" s="21"/>
+      <c r="T78" s="21"/>
+      <c r="U78" s="21"/>
+    </row>
+    <row r="79" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="N79" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="O79" s="23"/>
+      <c r="P79" s="23"/>
+      <c r="Q79" s="23"/>
+      <c r="R79" s="23"/>
+      <c r="S79" s="23"/>
+      <c r="T79" s="23"/>
+      <c r="U79" s="23"/>
+    </row>
+    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="N80" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="O80" s="20"/>
+      <c r="P80" s="20"/>
+      <c r="Q80" s="20"/>
+      <c r="R80" s="20"/>
+      <c r="S80" s="20"/>
+      <c r="T80" s="20"/>
+      <c r="U80" s="20"/>
+    </row>
+    <row r="81" spans="14:21" x14ac:dyDescent="0.3">
+      <c r="N81" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="O81" s="20"/>
+      <c r="P81" s="20"/>
+      <c r="Q81" s="20"/>
+      <c r="R81" s="20"/>
+      <c r="S81" s="20"/>
+      <c r="T81" s="20"/>
+      <c r="U81" s="20"/>
+    </row>
+    <row r="82" spans="14:21" x14ac:dyDescent="0.3">
+      <c r="N82" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="O82" s="20"/>
+      <c r="P82" s="20"/>
+      <c r="Q82" s="20"/>
+      <c r="R82" s="20"/>
+      <c r="S82" s="20"/>
+      <c r="T82" s="20"/>
+      <c r="U82" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="49">
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:L40"/>
+    <mergeCell ref="F45:L45"/>
+    <mergeCell ref="F46:L46"/>
+    <mergeCell ref="F39:L39"/>
+    <mergeCell ref="F35:L35"/>
+    <mergeCell ref="G36:L36"/>
+    <mergeCell ref="F37:L37"/>
+    <mergeCell ref="F38:L38"/>
+    <mergeCell ref="F30:L30"/>
+    <mergeCell ref="F41:L41"/>
+    <mergeCell ref="F42:L42"/>
+    <mergeCell ref="F44:L44"/>
+    <mergeCell ref="F43:L43"/>
+    <mergeCell ref="F31:L31"/>
+    <mergeCell ref="G32:L32"/>
+    <mergeCell ref="F33:L33"/>
+    <mergeCell ref="F34:L34"/>
+    <mergeCell ref="H25:L25"/>
+    <mergeCell ref="F26:L26"/>
+    <mergeCell ref="F27:L27"/>
+    <mergeCell ref="H28:L28"/>
+    <mergeCell ref="F29:L29"/>
+    <mergeCell ref="F20:L20"/>
+    <mergeCell ref="F21:L21"/>
+    <mergeCell ref="G22:L22"/>
+    <mergeCell ref="F23:L23"/>
+    <mergeCell ref="F24:L24"/>
+    <mergeCell ref="F15:L15"/>
+    <mergeCell ref="F16:L16"/>
+    <mergeCell ref="F17:L17"/>
+    <mergeCell ref="H18:L18"/>
+    <mergeCell ref="F19:L19"/>
+    <mergeCell ref="F10:L10"/>
+    <mergeCell ref="F11:L11"/>
+    <mergeCell ref="F12:L12"/>
+    <mergeCell ref="G14:L14"/>
+    <mergeCell ref="F13:L13"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A63:D63"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="F5:L5"/>
+    <mergeCell ref="F6:L6"/>
+    <mergeCell ref="G3:L3"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="F7:L7"/>
+    <mergeCell ref="G8:L8"/>
+    <mergeCell ref="F9:L9"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>